<commit_message>
Reformulando o código, usando classes.
</commit_message>
<xml_diff>
--- a/data/empuxo_TESTE_30_05_25.xlsx
+++ b/data/empuxo_TESTE_30_05_25.xlsx
@@ -24,18 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="21" uniqueCount="16">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="20" uniqueCount="15">
   <si>
     <t>Tempo [s]</t>
   </si>
   <si>
-    <t>Tempo/2 [s]</t>
-  </si>
-  <si>
     <t>Empuxo [N]</t>
-  </si>
-  <si>
-    <t>Fcalc</t>
   </si>
   <si>
     <t>Dt [m]</t>
@@ -72,6 +66,9 @@
   </si>
   <si>
     <t>Isp [s]</t>
+  </si>
+  <si>
+    <t>MEDIA</t>
   </si>
 </sst>
 </file>
@@ -880,7 +877,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="9.875" bestFit="1" customWidth="1"/>
@@ -903,53 +900,37 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="I1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="J1" t="s">
         <v>3</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>4</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>5</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>7</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>8</v>
-      </c>
-      <c r="N1" t="s">
-        <v>9</v>
-      </c>
-      <c r="O1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:15">
       <c r="A2">
-        <v>0.33100000000000002</v>
+        <v>0</v>
       </c>
       <c r="B2">
-        <v>0.16550000000000001</v>
-      </c>
-      <c r="C2">
-        <v>0.76</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>10.174329999999999</v>
-      </c>
+        <v>0.74</v>
+      </c>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
       <c r="I2">
         <v>1.2540000000000001E-2</v>
       </c>
@@ -974,25 +955,13 @@
     </row>
     <row r="3" spans="1:15">
       <c r="A3">
-        <v>0.44600000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="B3">
-        <v>0.223</v>
-      </c>
-      <c r="C3">
-        <v>0.75</v>
-      </c>
-      <c r="D3" s="2">
-        <f>(A3-A2)*(C3+C2)/2</f>
-        <v>8.6824999999999999E-2</v>
-      </c>
-      <c r="E3" s="2">
-        <f>(B3-B2)*(C3+C2)/2</f>
-        <v>4.34125E-2</v>
-      </c>
-      <c r="F3">
-        <v>10.174329999999999</v>
-      </c>
+        <v>0.73</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
       <c r="K3">
         <v>145325</v>
       </c>
@@ -1005,25 +974,13 @@
     </row>
     <row r="4" spans="1:15">
       <c r="A4">
-        <v>0.56000000000000005</v>
+        <v>0.2</v>
       </c>
       <c r="B4">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="C4">
-        <v>0.76</v>
-      </c>
-      <c r="D4" s="2">
-        <f t="shared" ref="D4:D28" si="0">(A4-A3)*(C4+C3)/2</f>
-        <v>8.6070000000000035E-2</v>
-      </c>
-      <c r="E4" s="2">
-        <f t="shared" ref="E4:E28" si="1">(B4-B3)*(C4+C3)/2</f>
-        <v>4.3035000000000018E-2</v>
-      </c>
-      <c r="F4">
-        <v>13.68004213</v>
-      </c>
+        <v>0.73</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
       <c r="K4">
         <v>167325</v>
       </c>
@@ -1036,24 +993,28 @@
     </row>
     <row r="5" spans="1:15">
       <c r="A5">
-        <v>0.66800000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="B5">
-        <v>0.33400000000000002</v>
-      </c>
-      <c r="C5">
-        <v>0.78</v>
-      </c>
-      <c r="D5" s="2">
-        <f t="shared" si="0"/>
-        <v>8.3159999999999984E-2</v>
-      </c>
-      <c r="E5" s="2">
-        <f t="shared" si="1"/>
-        <v>4.1579999999999992E-2</v>
-      </c>
-      <c r="F5">
-        <v>17.132090600000002</v>
+        <v>0.76</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" t="s">
+        <v>14</v>
       </c>
       <c r="K5">
         <v>189325</v>
@@ -1067,24 +1028,32 @@
     </row>
     <row r="6" spans="1:15">
       <c r="A6">
-        <v>0.74</v>
+        <v>0.4</v>
       </c>
       <c r="B6">
-        <v>0.37</v>
-      </c>
-      <c r="C6">
-        <v>2.09</v>
-      </c>
-      <c r="D6" s="2">
-        <f t="shared" si="0"/>
-        <v>0.10331999999999994</v>
-      </c>
-      <c r="E6" s="2">
-        <f t="shared" si="1"/>
-        <v>5.165999999999997E-2</v>
-      </c>
-      <c r="F6">
-        <v>13.68004213</v>
+        <v>0.75</v>
+      </c>
+      <c r="D6">
+        <f>SUMPRODUCT((A3:A45 - A2:A44), (B3:B45 + B2:B44)) / 2</f>
+        <v>293.57099999999997</v>
+      </c>
+      <c r="E6">
+        <v>0.34467826050420203</v>
+      </c>
+      <c r="F6" s="1">
+        <v>9.8066499999999994</v>
+      </c>
+      <c r="G6">
+        <f>E6*F6</f>
+        <v>3.3801390633735324</v>
+      </c>
+      <c r="H6">
+        <f>D6/G6</f>
+        <v>86.851752101288625</v>
+      </c>
+      <c r="I6">
+        <f>AVERAGE(B12:B31)</f>
+        <v>144.74950000000004</v>
       </c>
       <c r="K6">
         <v>167325</v>
@@ -1098,24 +1067,25 @@
     </row>
     <row r="7" spans="1:15">
       <c r="A7">
-        <v>0.84899999999999998</v>
+        <v>0.5</v>
       </c>
       <c r="B7">
-        <v>0.42449999999999999</v>
-      </c>
-      <c r="C7">
-        <v>12.1</v>
-      </c>
-      <c r="D7" s="2">
-        <f t="shared" si="0"/>
-        <v>0.7733549999999999</v>
-      </c>
-      <c r="E7" s="2">
-        <f t="shared" si="1"/>
-        <v>0.38667749999999995</v>
-      </c>
-      <c r="F7">
-        <v>32.785685030000003</v>
+        <v>0.76</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" t="s">
+        <v>13</v>
       </c>
       <c r="K7">
         <v>288325</v>
@@ -1129,24 +1099,28 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8">
-        <v>0.89500000000000002</v>
+        <v>0.6</v>
       </c>
       <c r="B8">
-        <v>0.44750000000000001</v>
-      </c>
-      <c r="C8">
-        <v>12.1</v>
-      </c>
-      <c r="D8" s="2">
-        <f t="shared" si="0"/>
-        <v>0.55660000000000043</v>
-      </c>
-      <c r="E8" s="2">
-        <f t="shared" si="1"/>
-        <v>0.27830000000000021</v>
+        <v>0.78</v>
+      </c>
+      <c r="D8">
+        <f>SUM(E2:E28)</f>
+        <v>0.68935652100840406</v>
+      </c>
+      <c r="E8">
+        <v>0.34467826050420203</v>
       </c>
       <c r="F8">
-        <v>32.785685030000003</v>
+        <v>9.8066499999999994</v>
+      </c>
+      <c r="G8">
+        <f>E8*F8</f>
+        <v>3.3801390633735324</v>
+      </c>
+      <c r="H8">
+        <f>D8/G8</f>
+        <v>0.20394324259558566</v>
       </c>
       <c r="K8">
         <v>288325</v>
@@ -1160,25 +1134,13 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9">
-        <v>0.95899999999999996</v>
+        <v>0.7</v>
       </c>
       <c r="B9">
-        <v>0.47949999999999998</v>
-      </c>
-      <c r="C9">
-        <v>24.87</v>
-      </c>
-      <c r="D9" s="2">
-        <f t="shared" si="0"/>
-        <v>1.183039999999999</v>
-      </c>
-      <c r="E9" s="2">
-        <f t="shared" si="1"/>
-        <v>0.59151999999999949</v>
-      </c>
-      <c r="F9">
-        <v>54.352659869999997</v>
-      </c>
+        <v>2.09</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
       <c r="K9">
         <v>420325</v>
       </c>
@@ -1191,25 +1153,13 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10">
-        <v>1.05</v>
+        <v>0.8</v>
       </c>
       <c r="B10">
-        <v>0.52500000000000002</v>
-      </c>
-      <c r="C10">
-        <v>35.6</v>
-      </c>
-      <c r="D10" s="2">
-        <f t="shared" si="0"/>
-        <v>2.7513850000000022</v>
-      </c>
-      <c r="E10" s="2">
-        <f t="shared" si="1"/>
-        <v>1.3756925000000011</v>
-      </c>
-      <c r="F10">
-        <v>63.545122650000003</v>
-      </c>
+        <v>12.1</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
       <c r="K10">
         <v>475325</v>
       </c>
@@ -1222,25 +1172,13 @@
     </row>
     <row r="11" spans="1:15">
       <c r="A11">
-        <v>1.1259999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="B11">
-        <v>0.56299999999999994</v>
-      </c>
-      <c r="C11">
-        <v>35.6</v>
-      </c>
-      <c r="D11" s="2">
-        <f t="shared" si="0"/>
-        <v>2.7055999999999947</v>
-      </c>
-      <c r="E11" s="2">
-        <f t="shared" si="1"/>
-        <v>1.3527999999999973</v>
-      </c>
-      <c r="F11">
-        <v>63.545122650000003</v>
-      </c>
+        <v>12.1</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
       <c r="K11">
         <v>475325</v>
       </c>
@@ -1253,25 +1191,13 @@
     </row>
     <row r="12" spans="1:15">
       <c r="A12">
-        <v>1.2589999999999999</v>
+        <v>1</v>
       </c>
       <c r="B12">
-        <v>0.62949999999999995</v>
-      </c>
-      <c r="C12">
-        <v>71.59</v>
-      </c>
-      <c r="D12" s="2">
-        <f t="shared" si="0"/>
-        <v>7.1281350000000003</v>
-      </c>
-      <c r="E12" s="2">
-        <f t="shared" si="1"/>
-        <v>3.5640675000000002</v>
-      </c>
-      <c r="F12">
-        <v>99.299140879999996</v>
-      </c>
+        <v>24.87</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
       <c r="K12">
         <v>684325</v>
       </c>
@@ -1284,25 +1210,13 @@
     </row>
     <row r="13" spans="1:15">
       <c r="A13">
-        <v>1.327</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="B13">
-        <v>0.66349999999999998</v>
-      </c>
-      <c r="C13">
-        <v>71.59</v>
-      </c>
-      <c r="D13" s="2">
-        <f t="shared" si="0"/>
-        <v>4.8681200000000047</v>
-      </c>
-      <c r="E13" s="2">
-        <f t="shared" si="1"/>
-        <v>2.4340600000000023</v>
-      </c>
-      <c r="F13">
-        <v>99.299140879999996</v>
-      </c>
+        <v>35.6</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
       <c r="K13">
         <v>684325</v>
       </c>
@@ -1315,25 +1229,13 @@
     </row>
     <row r="14" spans="1:15">
       <c r="A14">
-        <v>1.4850000000000001</v>
+        <v>1.2</v>
       </c>
       <c r="B14">
-        <v>0.74250000000000005</v>
-      </c>
-      <c r="C14">
-        <v>183.83</v>
-      </c>
-      <c r="D14" s="2">
-        <f t="shared" si="0"/>
-        <v>20.178180000000019</v>
-      </c>
-      <c r="E14" s="2">
-        <f t="shared" si="1"/>
-        <v>10.089090000000009</v>
-      </c>
-      <c r="F14">
-        <v>223.40657490000001</v>
-      </c>
+        <v>35.6</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
       <c r="K14">
         <v>1377325</v>
       </c>
@@ -1346,25 +1248,13 @@
     </row>
     <row r="15" spans="1:15">
       <c r="A15">
-        <v>1.56</v>
+        <v>1.3</v>
       </c>
       <c r="B15">
-        <v>0.78</v>
-      </c>
-      <c r="C15">
-        <v>200.54</v>
-      </c>
-      <c r="D15" s="2">
-        <f t="shared" si="0"/>
-        <v>14.413874999999992</v>
-      </c>
-      <c r="E15" s="2">
-        <f t="shared" si="1"/>
-        <v>7.206937499999996</v>
-      </c>
-      <c r="F15">
-        <v>255.766727</v>
-      </c>
+        <v>71.59</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
       <c r="K15">
         <v>1553325</v>
       </c>
@@ -1377,25 +1267,13 @@
     </row>
     <row r="16" spans="1:15">
       <c r="A16">
-        <v>1.6479999999999999</v>
+        <v>1.4</v>
       </c>
       <c r="B16">
-        <v>0.82399999999999995</v>
-      </c>
-      <c r="C16">
-        <v>224.49</v>
-      </c>
-      <c r="D16" s="2">
-        <f t="shared" si="0"/>
-        <v>18.701319999999967</v>
-      </c>
-      <c r="E16" s="2">
-        <f t="shared" si="1"/>
-        <v>9.3506599999999835</v>
-      </c>
-      <c r="F16">
-        <v>284.27687150000003</v>
-      </c>
+        <v>71.59</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
       <c r="K16">
         <v>1707325</v>
       </c>
@@ -1408,25 +1286,13 @@
     </row>
     <row r="17" spans="1:13">
       <c r="A17">
-        <v>1.9379999999999999</v>
+        <v>1.5</v>
       </c>
       <c r="B17">
-        <v>0.96899999999999997</v>
-      </c>
-      <c r="C17">
-        <v>230.57</v>
-      </c>
-      <c r="D17" s="2">
-        <f t="shared" si="0"/>
-        <v>65.983700000000013</v>
-      </c>
-      <c r="E17" s="2">
-        <f t="shared" si="1"/>
-        <v>32.991850000000007</v>
-      </c>
-      <c r="F17">
-        <v>278.15345159999998</v>
-      </c>
+        <v>183.83</v>
+      </c>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
       <c r="K17">
         <v>1674325</v>
       </c>
@@ -1439,25 +1305,13 @@
     </row>
     <row r="18" spans="1:13">
       <c r="A18">
-        <v>2.238</v>
+        <v>1.6</v>
       </c>
       <c r="B18">
-        <v>1.119</v>
-      </c>
-      <c r="C18">
-        <v>240.23</v>
-      </c>
-      <c r="D18" s="2">
-        <f t="shared" si="0"/>
-        <v>70.62</v>
-      </c>
-      <c r="E18" s="2">
-        <f t="shared" si="1"/>
-        <v>35.31</v>
-      </c>
-      <c r="F18">
-        <v>282.23490850000002</v>
-      </c>
+        <v>200.54</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
       <c r="K18">
         <v>1696325</v>
       </c>
@@ -1470,25 +1324,13 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19">
-        <v>2.5510000000000002</v>
+        <v>1.7</v>
       </c>
       <c r="B19">
-        <v>1.2755000000000001</v>
-      </c>
-      <c r="C19">
-        <v>237.18</v>
-      </c>
-      <c r="D19" s="2">
-        <f t="shared" si="0"/>
-        <v>74.714665000000039</v>
-      </c>
-      <c r="E19" s="2">
-        <f t="shared" si="1"/>
-        <v>37.35733250000002</v>
-      </c>
-      <c r="F19">
-        <v>282.23490850000002</v>
-      </c>
+        <v>224.49</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
       <c r="K19">
         <v>1696325</v>
       </c>
@@ -1501,25 +1343,13 @@
     </row>
     <row r="20" spans="1:13">
       <c r="A20">
-        <v>3.0009999999999999</v>
+        <v>1.8</v>
       </c>
       <c r="B20">
-        <v>1.5004999999999999</v>
-      </c>
-      <c r="C20">
-        <v>237.18</v>
-      </c>
-      <c r="D20" s="2">
-        <f t="shared" si="0"/>
-        <v>106.73099999999994</v>
-      </c>
-      <c r="E20" s="2">
-        <f t="shared" si="1"/>
-        <v>53.365499999999969</v>
-      </c>
-      <c r="F20">
-        <v>282.23490850000002</v>
-      </c>
+        <v>230.57</v>
+      </c>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
       <c r="K20">
         <v>1696325</v>
       </c>
@@ -1532,25 +1362,13 @@
     </row>
     <row r="21" spans="1:13">
       <c r="A21">
-        <v>3.3010000000000002</v>
+        <v>1.9</v>
       </c>
       <c r="B21">
-        <v>1.6505000000000001</v>
-      </c>
-      <c r="C21">
-        <v>222.61</v>
-      </c>
-      <c r="D21" s="2">
-        <f t="shared" si="0"/>
-        <v>68.968500000000063</v>
-      </c>
-      <c r="E21" s="2">
-        <f t="shared" si="1"/>
-        <v>34.484250000000031</v>
-      </c>
-      <c r="F21">
-        <v>267.96454640000002</v>
-      </c>
+        <v>240.23</v>
+      </c>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
       <c r="K21">
         <v>1619325</v>
       </c>
@@ -1563,25 +1381,13 @@
     </row>
     <row r="22" spans="1:13">
       <c r="A22">
-        <v>3.5950000000000002</v>
+        <v>2</v>
       </c>
       <c r="B22">
-        <v>1.7975000000000001</v>
-      </c>
-      <c r="C22">
-        <v>207.76</v>
-      </c>
-      <c r="D22" s="2">
-        <f t="shared" si="0"/>
-        <v>63.264390000000006</v>
-      </c>
-      <c r="E22" s="2">
-        <f t="shared" si="1"/>
-        <v>31.632195000000003</v>
-      </c>
-      <c r="F22">
-        <v>257.7974443</v>
-      </c>
+        <v>237.18</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
       <c r="K22">
         <v>1564325</v>
       </c>
@@ -1594,25 +1400,13 @@
     </row>
     <row r="23" spans="1:13">
       <c r="A23">
-        <v>3.9220000000000002</v>
+        <v>2.1</v>
       </c>
       <c r="B23">
-        <v>1.9610000000000001</v>
-      </c>
-      <c r="C23">
-        <v>207.76</v>
-      </c>
-      <c r="D23" s="2">
-        <f t="shared" si="0"/>
-        <v>67.937519999999992</v>
-      </c>
-      <c r="E23" s="2">
-        <f t="shared" si="1"/>
-        <v>33.968759999999996</v>
-      </c>
-      <c r="F23">
-        <v>257.7974443</v>
-      </c>
+        <v>237.18</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
       <c r="K23">
         <v>1564325</v>
       </c>
@@ -1625,25 +1419,13 @@
     </row>
     <row r="24" spans="1:13">
       <c r="A24">
-        <v>4.25</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="B24">
-        <v>2.125</v>
-      </c>
-      <c r="C24">
-        <v>176.59</v>
-      </c>
-      <c r="D24" s="2">
-        <f t="shared" si="0"/>
-        <v>63.033399999999972</v>
-      </c>
-      <c r="E24" s="2">
-        <f t="shared" si="1"/>
-        <v>31.516699999999986</v>
-      </c>
-      <c r="F24">
-        <v>215.3579135</v>
-      </c>
+        <v>222.61</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
       <c r="K24">
         <v>1333325</v>
       </c>
@@ -1656,25 +1438,13 @@
     </row>
     <row r="25" spans="1:13">
       <c r="A25">
-        <v>4.6909999999999998</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="B25">
-        <v>2.3454999999999999</v>
-      </c>
-      <c r="C25">
-        <v>176.59</v>
-      </c>
-      <c r="D25" s="2">
-        <f t="shared" si="0"/>
-        <v>77.876189999999966</v>
-      </c>
-      <c r="E25" s="2">
-        <f t="shared" si="1"/>
-        <v>38.938094999999983</v>
-      </c>
-      <c r="F25">
-        <v>215.3579135</v>
-      </c>
+        <v>207.76</v>
+      </c>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
       <c r="K25">
         <v>1333325</v>
       </c>
@@ -1687,25 +1457,13 @@
     </row>
     <row r="26" spans="1:13">
       <c r="A26">
-        <v>4.9729999999999999</v>
+        <v>2.4</v>
       </c>
       <c r="B26">
-        <v>2.4864999999999999</v>
-      </c>
-      <c r="C26">
-        <v>71.09</v>
-      </c>
-      <c r="D26" s="2">
-        <f t="shared" si="0"/>
-        <v>34.922880000000006</v>
-      </c>
-      <c r="E26" s="2">
-        <f t="shared" si="1"/>
-        <v>17.461440000000003</v>
-      </c>
-      <c r="F26">
-        <v>108.8822033</v>
-      </c>
+        <v>207.76</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
       <c r="K26">
         <v>739325</v>
       </c>
@@ -1718,25 +1476,13 @@
     </row>
     <row r="27" spans="1:13">
       <c r="A27">
-        <v>5.2990000000000004</v>
+        <v>2.5</v>
       </c>
       <c r="B27">
-        <v>2.6495000000000002</v>
-      </c>
-      <c r="C27">
-        <v>19.66</v>
-      </c>
-      <c r="D27" s="2">
-        <f t="shared" si="0"/>
-        <v>14.792250000000024</v>
-      </c>
-      <c r="E27" s="2">
-        <f t="shared" si="1"/>
-        <v>7.3961250000000121</v>
-      </c>
-      <c r="F27">
-        <v>43.473566079999998</v>
-      </c>
+        <v>176.59</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
       <c r="K27">
         <v>354325</v>
       </c>
@@ -1749,25 +1495,13 @@
     </row>
     <row r="28" spans="1:13">
       <c r="A28">
-        <v>5.62</v>
+        <v>2.6</v>
       </c>
       <c r="B28">
-        <v>2.81</v>
-      </c>
-      <c r="C28">
-        <v>19.66</v>
-      </c>
-      <c r="D28" s="2">
-        <f t="shared" si="0"/>
-        <v>6.3108599999999946</v>
-      </c>
-      <c r="E28" s="2">
-        <f t="shared" si="1"/>
-        <v>3.1554299999999973</v>
-      </c>
-      <c r="F28">
-        <v>43.473566079999998</v>
-      </c>
+        <v>176.59</v>
+      </c>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
       <c r="K28">
         <v>354325</v>
       </c>
@@ -1778,78 +1512,132 @@
         <v>0.253</v>
       </c>
     </row>
+    <row r="29" spans="1:13">
+      <c r="A29">
+        <v>2.7</v>
+      </c>
+      <c r="B29">
+        <v>71.09</v>
+      </c>
+    </row>
     <row r="30" spans="1:13">
-      <c r="A30" t="s">
-        <v>11</v>
-      </c>
-      <c r="B30" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30" t="s">
-        <v>13</v>
-      </c>
-      <c r="D30" t="s">
-        <v>14</v>
-      </c>
-      <c r="E30" t="s">
-        <v>15</v>
+      <c r="A30">
+        <v>2.8</v>
+      </c>
+      <c r="B30">
+        <v>19.66</v>
       </c>
     </row>
     <row r="31" spans="1:13">
       <c r="A31">
-        <f>SUM(D2:D28)</f>
-        <v>788.77433999999994</v>
+        <v>2.9</v>
       </c>
       <c r="B31">
-        <v>0.34467826050420203</v>
-      </c>
-      <c r="C31" s="1">
-        <v>9.8066499999999994</v>
-      </c>
-      <c r="D31">
-        <f>B31*C31</f>
-        <v>3.3801390633735324</v>
-      </c>
-      <c r="E31">
-        <f>A31/D31</f>
-        <v>233.35558839782388</v>
+        <v>19.66</v>
       </c>
     </row>
     <row r="32" spans="1:13">
-      <c r="A32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B32" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" t="s">
-        <v>14</v>
-      </c>
-      <c r="E32" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="A32">
+        <v>3</v>
+      </c>
+      <c r="B32">
+        <v>4.63</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
       <c r="A33">
-        <f>SUM(E2:E28)</f>
-        <v>394.38716999999997</v>
+        <v>3.1</v>
       </c>
       <c r="B33">
-        <v>0.34467826050420203</v>
-      </c>
-      <c r="C33">
-        <v>9.8066499999999994</v>
-      </c>
-      <c r="D33">
-        <f>B33*C33</f>
-        <v>3.3801390633735324</v>
-      </c>
-      <c r="E33">
-        <f>A33/D33</f>
-        <v>116.67779419891194</v>
+        <v>3.08</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34">
+        <v>3.2</v>
+      </c>
+      <c r="B34">
+        <v>3.08</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35">
+        <v>3.3</v>
+      </c>
+      <c r="B35">
+        <v>2.61</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36">
+        <v>3.4</v>
+      </c>
+      <c r="B36">
+        <v>2.61</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37">
+        <v>3.5</v>
+      </c>
+      <c r="B37">
+        <v>2.58</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38">
+        <v>3.6</v>
+      </c>
+      <c r="B38">
+        <v>2.46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39">
+        <v>3.7</v>
+      </c>
+      <c r="B39">
+        <v>1.56</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40">
+        <v>3.8</v>
+      </c>
+      <c r="B40">
+        <v>1.1299999999999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41">
+        <v>3.9</v>
+      </c>
+      <c r="B41">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42">
+        <v>4</v>
+      </c>
+      <c r="B42">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B43">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44">
+        <v>4.2</v>
+      </c>
+      <c r="B44">
+        <v>0.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>